<commit_message>
avance primera version funcional en produccion
</commit_message>
<xml_diff>
--- a/temp_mhr/desasignar_53069883.xlsx
+++ b/temp_mhr/desasignar_53069883.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -470,24 +470,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>700128118</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>53069883</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>501108307</t>
+          <t>700179979</t>
         </is>
       </c>
     </row>

</xml_diff>